<commit_message>
changements mineurs (documentation, commentaires)
</commit_message>
<xml_diff>
--- a/data/01_export/hashFiles.xlsx
+++ b/data/01_export/hashFiles.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,18 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>2026-05-18 11:59:18.764205</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2c9aca039b34ade067579dde2670173f</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-19 11:52:18.896548</t>
         </is>
       </c>
     </row>

</xml_diff>